<commit_message>
Mark ExtraCash installment as confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EPNKNk7kASs5DQVTsUv5rh
</commit_message>
<xml_diff>
--- a/finanzas/libro-caja-deuda.xlsx
+++ b/finanzas/libro-caja-deuda.xlsx
@@ -136,8 +136,8 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3092,12 +3092,12 @@
           <t>Cuota mensual (24 meses)</t>
         </is>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="18" t="n">
         <v>534.5599999999999</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Estimado: 441.38 x 10,900/9,000. Confirmar en la app</t>
+          <t>Confirmado en la app Interbank (simulación 10,900 a 24 meses)</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3107,7 @@
           <t>TEA</t>
         </is>
       </c>
-      <c r="B14" s="21" t="n">
+      <c r="B14" s="20" t="n">
         <v>0.1663</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -3122,7 +3122,7 @@
           <t>Seguro desgravamen incluido en la cuota</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n">
+      <c r="B15" s="21" t="n">
         <v>3.55</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3224,7 +3224,7 @@
           <t>Interés residual + seguro (estado 21/10)</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="21" t="n">
         <v>275</v>
       </c>
       <c r="C23" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add monthly building maintenance (Oct-Dec) to debt ledger
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EPNKNk7kASs5DQVTsUv5rh
</commit_message>
<xml_diff>
--- a/finanzas/libro-caja-deuda.xlsx
+++ b/finanzas/libro-caja-deuda.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Libro de caja - Escenario A2 (ExtraCash S/ 10,900)</t>
+          <t>Libro de caja - Escenario A2 (ExtraCash S/ 10,900) - v2 con mantenimiento</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="9">
-        <f>Supuestos!$C$29</f>
+        <f>Supuestos!$C$31</f>
         <v/>
       </c>
       <c r="F10" s="9">
@@ -726,7 +726,7 @@
       </c>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="9">
-        <f>Supuestos!$C$30</f>
+        <f>Supuestos!$C$32</f>
         <v/>
       </c>
       <c r="F11" s="9">
@@ -751,7 +751,7 @@
       </c>
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9">
-        <f>Supuestos!$C$31</f>
+        <f>Supuestos!$C$33</f>
         <v/>
       </c>
       <c r="F12" s="9">
@@ -776,7 +776,7 @@
       </c>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="9">
-        <f>Supuestos!$C$32</f>
+        <f>Supuestos!$C$34</f>
         <v/>
       </c>
       <c r="F13" s="9">
@@ -801,7 +801,7 @@
       </c>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9">
-        <f>Supuestos!$C$33</f>
+        <f>Supuestos!$C$35</f>
         <v/>
       </c>
       <c r="F14" s="9">
@@ -810,89 +810,89 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11">
+      <c r="A15" s="7">
+        <f>'Plan mensual'!$A$5+9</f>
+        <v/>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Mantenimiento + agua (Yape)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Gasto fijo</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9">
+        <f>IF('Plan mensual'!$A$5&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>F14+D15-E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
         <f>EOMONTH('Plan mensual'!$A$5,0)</f>
         <v/>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>SALDO FINAL DEL MES</t>
         </is>
       </c>
-      <c r="C15" s="12">
+      <c r="C16" s="12">
         <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H5,"#,##0.00")</f>
         <v/>
       </c>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13">
-        <f>F14</f>
-        <v/>
-      </c>
-      <c r="H15" s="14">
-        <f>IF(ABS(F15-'Plan mensual'!K5)&lt;0.01,"OK","Revisar")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13">
+        <f>F15</f>
+        <v/>
+      </c>
+      <c r="H16" s="14">
+        <f>IF(ABS(F16-'Plan mensual'!K5)&lt;0.01,"OK","Revisar")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Noviembre 2026</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7">
-        <f>'Plan mensual'!$A$6-1</f>
-        <v/>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Sueldo Simtryx</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D18" s="10">
-        <f>'Plan mensual'!C6</f>
-        <v/>
-      </c>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9">
-        <f>F15+D18-E18</f>
-        <v/>
-      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7">
-        <f>'Plan mensual'!$A$6+14</f>
+        <f>'Plan mensual'!$A$6-1</f>
         <v/>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior) + pendientes + interés residual</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="10">
-        <f>'Plan mensual'!F6</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D19" s="10">
+        <f>'Plan mensual'!C6</f>
+        <v/>
+      </c>
+      <c r="E19" s="9" t="n"/>
       <c r="F19" s="9">
-        <f>F18+D19-E19</f>
+        <f>F16+D19-E19</f>
         <v/>
       </c>
     </row>
@@ -903,17 +903,17 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior) + pendientes + interés residual</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="10">
-        <f>'Plan mensual'!G6</f>
+        <f>'Plan mensual'!F6</f>
         <v/>
       </c>
       <c r="F20" s="9">
@@ -923,12 +923,12 @@
     </row>
     <row r="21">
       <c r="A21" s="7">
-        <f>'Plan mensual'!$A$6+21</f>
+        <f>'Plan mensual'!$A$6+14</f>
         <v/>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="10">
-        <f>'Plan mensual'!J6</f>
+        <f>'Plan mensual'!G6</f>
         <v/>
       </c>
       <c r="F21" s="9">
@@ -948,22 +948,22 @@
     </row>
     <row r="22">
       <c r="A22" s="7">
-        <f>EOMONTH('Plan mensual'!$A$6,0)</f>
+        <f>'Plan mensual'!$A$6+21</f>
         <v/>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9">
-        <f>Supuestos!$B$29</f>
+      <c r="E22" s="10">
+        <f>'Plan mensual'!J6</f>
         <v/>
       </c>
       <c r="F22" s="9">
@@ -978,7 +978,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9">
-        <f>Supuestos!$B$30</f>
+        <f>Supuestos!$B$31</f>
         <v/>
       </c>
       <c r="F23" s="9">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Delivery (total del mes)</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9">
-        <f>Supuestos!$B$31</f>
+        <f>Supuestos!$B$32</f>
         <v/>
       </c>
       <c r="F24" s="9">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9">
-        <f>Supuestos!$B$32</f>
+        <f>Supuestos!$B$33</f>
         <v/>
       </c>
       <c r="F25" s="9">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9">
-        <f>Supuestos!$B$33</f>
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F26" s="9">
@@ -1072,135 +1072,135 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11">
+      <c r="A27" s="7">
         <f>EOMONTH('Plan mensual'!$A$6,0)</f>
         <v/>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Contador Luxr (total del mes)</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9">
+        <f>Supuestos!$B$35</f>
+        <v/>
+      </c>
+      <c r="F27" s="9">
+        <f>F26+D27-E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7">
+        <f>'Plan mensual'!$A$6+9</f>
+        <v/>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Mantenimiento + agua (Yape)</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Gasto fijo</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="9">
+        <f>IF('Plan mensual'!$A$6&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="F28" s="9">
+        <f>F27+D28-E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11">
+        <f>EOMONTH('Plan mensual'!$A$6,0)</f>
+        <v/>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>SALDO FINAL DEL MES</t>
         </is>
       </c>
-      <c r="C27" s="12">
+      <c r="C29" s="12">
         <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H6,"#,##0.00")</f>
         <v/>
       </c>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13">
-        <f>F26</f>
-        <v/>
-      </c>
-      <c r="H27" s="14">
-        <f>IF(ABS(F27-'Plan mensual'!K6)&lt;0.01,"OK","Revisar")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13">
+        <f>F28</f>
+        <v/>
+      </c>
+      <c r="H29" s="14">
+        <f>IF(ABS(F29-'Plan mensual'!K6)&lt;0.01,"OK","Revisar")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Diciembre 2026</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="7">
-        <f>'Plan mensual'!$A$7-1</f>
-        <v/>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>Sueldo Simtryx</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D30" s="10">
-        <f>'Plan mensual'!C7</f>
-        <v/>
-      </c>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9">
-        <f>F27+D30-E30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7">
-        <f>'Plan mensual'!$A$7+14</f>
-        <v/>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="10">
-        <f>'Plan mensual'!F7</f>
-        <v/>
-      </c>
-      <c r="F31" s="9">
-        <f>F30+D31-E31</f>
-        <v/>
-      </c>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7">
-        <f>'Plan mensual'!$A$7+14</f>
+        <f>'Plan mensual'!$A$7-1</f>
         <v/>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="10">
-        <f>'Plan mensual'!G7</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D32" s="10">
+        <f>'Plan mensual'!C7</f>
+        <v/>
+      </c>
+      <c r="E32" s="9" t="n"/>
       <c r="F32" s="9">
-        <f>F31+D32-E32</f>
+        <f>F29+D32-E32</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7">
-        <f>'Plan mensual'!$A$7+21</f>
+        <f>'Plan mensual'!$A$7+14</f>
         <v/>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="10">
-        <f>'Plan mensual'!J7</f>
+        <f>'Plan mensual'!F7</f>
         <v/>
       </c>
       <c r="F33" s="9">
@@ -1210,22 +1210,22 @@
     </row>
     <row r="34">
       <c r="A34" s="7">
-        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
+        <f>'Plan mensual'!$A$7+14</f>
         <v/>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D34" s="9" t="n"/>
-      <c r="E34" s="9">
-        <f>Supuestos!$B$29</f>
+      <c r="E34" s="10">
+        <f>'Plan mensual'!G7</f>
         <v/>
       </c>
       <c r="F34" s="9">
@@ -1235,22 +1235,22 @@
     </row>
     <row r="35">
       <c r="A35" s="7">
-        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
+        <f>'Plan mensual'!$A$7+21</f>
         <v/>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D35" s="9" t="n"/>
-      <c r="E35" s="9">
-        <f>Supuestos!$B$30</f>
+      <c r="E35" s="10">
+        <f>'Plan mensual'!J7</f>
         <v/>
       </c>
       <c r="F35" s="9">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Delivery (total del mes)</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
@@ -1334,160 +1334,160 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11">
+      <c r="A39" s="7">
         <f>EOMONTH('Plan mensual'!$A$7,0)</f>
         <v/>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Otros (total del mes)</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9">
+        <f>Supuestos!$B$34</f>
+        <v/>
+      </c>
+      <c r="F39" s="9">
+        <f>F38+D39-E39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7">
+        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
+        <v/>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Contador Luxr (total del mes)</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9">
+        <f>Supuestos!$B$35</f>
+        <v/>
+      </c>
+      <c r="F40" s="9">
+        <f>F39+D40-E40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7">
+        <f>'Plan mensual'!$A$7+9</f>
+        <v/>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Mantenimiento + agua (Yape)</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Gasto fijo</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9">
+        <f>IF('Plan mensual'!$A$7&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="F41" s="9">
+        <f>F40+D41-E41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11">
+        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
+        <v/>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>SALDO FINAL DEL MES</t>
         </is>
       </c>
-      <c r="C39" s="12">
+      <c r="C42" s="12">
         <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H7,"#,##0.00")</f>
         <v/>
       </c>
-      <c r="D39" s="13" t="n"/>
-      <c r="E39" s="13" t="n"/>
-      <c r="F39" s="13">
-        <f>F38</f>
-        <v/>
-      </c>
-      <c r="H39" s="14">
-        <f>IF(ABS(F39-'Plan mensual'!K7)&lt;0.01,"OK","Revisar")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="D42" s="13" t="n"/>
+      <c r="E42" s="13" t="n"/>
+      <c r="F42" s="13">
+        <f>F41</f>
+        <v/>
+      </c>
+      <c r="H42" s="14">
+        <f>IF(ABS(F42-'Plan mensual'!K7)&lt;0.01,"OK","Revisar")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>Enero 2027</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="7">
-        <f>'Plan mensual'!$A$8-1</f>
-        <v/>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Sueldo Simtryx</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D42" s="10">
-        <f>'Plan mensual'!C8</f>
-        <v/>
-      </c>
-      <c r="E42" s="9" t="n"/>
-      <c r="F42" s="9">
-        <f>F39+D42-E42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="7">
-        <f>'Plan mensual'!$A$8+14</f>
-        <v/>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="10">
-        <f>'Plan mensual'!F8</f>
-        <v/>
-      </c>
-      <c r="F43" s="9">
-        <f>F42+D43-E43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="7">
-        <f>'Plan mensual'!$A$8+14</f>
-        <v/>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>Cuota ExtraCash</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D44" s="9" t="n"/>
-      <c r="E44" s="10">
-        <f>'Plan mensual'!G8</f>
-        <v/>
-      </c>
-      <c r="F44" s="9">
-        <f>F43+D44-E44</f>
-        <v/>
-      </c>
+      <c r="B44" s="6" t="n"/>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7">
-        <f>'Plan mensual'!$A$8+21</f>
+        <f>'Plan mensual'!$A$8-1</f>
         <v/>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="n"/>
-      <c r="E45" s="10">
-        <f>'Plan mensual'!J8</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D45" s="10">
+        <f>'Plan mensual'!C8</f>
+        <v/>
+      </c>
+      <c r="E45" s="9" t="n"/>
       <c r="F45" s="9">
-        <f>F44+D45-E45</f>
+        <f>F42+D45-E45</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7">
-        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
+        <f>'Plan mensual'!$A$8+14</f>
         <v/>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D46" s="9" t="n"/>
-      <c r="E46" s="9">
-        <f>Supuestos!$B$29</f>
+      <c r="E46" s="10">
+        <f>'Plan mensual'!F8</f>
         <v/>
       </c>
       <c r="F46" s="9">
@@ -1497,22 +1497,22 @@
     </row>
     <row r="47">
       <c r="A47" s="7">
-        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
+        <f>'Plan mensual'!$A$8+14</f>
         <v/>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9">
-        <f>Supuestos!$B$30</f>
+      <c r="E47" s="10">
+        <f>'Plan mensual'!G8</f>
         <v/>
       </c>
       <c r="F47" s="9">
@@ -1522,22 +1522,22 @@
     </row>
     <row r="48">
       <c r="A48" s="7">
-        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
+        <f>'Plan mensual'!$A$8+21</f>
         <v/>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D48" s="9" t="n"/>
-      <c r="E48" s="9">
-        <f>Supuestos!$B$31</f>
+      <c r="E48" s="10">
+        <f>'Plan mensual'!J8</f>
         <v/>
       </c>
       <c r="F48" s="9">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="9">
-        <f>Supuestos!$B$32</f>
+        <f>Supuestos!$B$31</f>
         <v/>
       </c>
       <c r="F49" s="9">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Delivery (total del mes)</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="D50" s="9" t="n"/>
       <c r="E50" s="9">
-        <f>Supuestos!$B$33</f>
+        <f>Supuestos!$B$32</f>
         <v/>
       </c>
       <c r="F50" s="9">
@@ -1596,185 +1596,185 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="11">
+      <c r="A51" s="7">
         <f>EOMONTH('Plan mensual'!$A$8,0)</f>
         <v/>
       </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C51" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H8,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D51" s="13" t="n"/>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="13">
-        <f>F50</f>
-        <v/>
-      </c>
-      <c r="H51" s="14">
-        <f>IF(ABS(F51-'Plan mensual'!K8)&lt;0.01,"OK","Revisar")</f>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Taxis (total del mes)</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="n"/>
+      <c r="E51" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
+      <c r="F51" s="9">
+        <f>F50+D51-E51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7">
+        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
+        <v/>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Otros (total del mes)</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="9">
+        <f>Supuestos!$B$34</f>
+        <v/>
+      </c>
+      <c r="F52" s="9">
+        <f>F51+D52-E52</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Febrero 2027</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
+      <c r="A53" s="7">
+        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
+        <v/>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Contador Luxr (total del mes)</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="9">
+        <f>Supuestos!$B$35</f>
+        <v/>
+      </c>
+      <c r="F53" s="9">
+        <f>F52+D53-E53</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7">
-        <f>'Plan mensual'!$A$9-1</f>
+        <f>'Plan mensual'!$A$8+9</f>
         <v/>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D54" s="10">
-        <f>'Plan mensual'!C9</f>
-        <v/>
-      </c>
-      <c r="E54" s="9" t="n"/>
+          <t>Gasto fijo</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n"/>
+      <c r="E54" s="9">
+        <f>IF('Plan mensual'!$A$8&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <v/>
+      </c>
       <c r="F54" s="9">
-        <f>F51+D54-E54</f>
+        <f>F53+D54-E54</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7">
-        <f>'Plan mensual'!$A$9+14</f>
-        <v/>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="D55" s="9" t="n"/>
-      <c r="E55" s="10">
-        <f>'Plan mensual'!F9</f>
-        <v/>
-      </c>
-      <c r="F55" s="9">
-        <f>F54+D55-E55</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7">
-        <f>'Plan mensual'!$A$9+14</f>
-        <v/>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>Cuota ExtraCash</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D56" s="9" t="n"/>
-      <c r="E56" s="10">
-        <f>'Plan mensual'!G9</f>
-        <v/>
-      </c>
-      <c r="F56" s="9">
-        <f>F55+D56-E56</f>
+      <c r="A55" s="11">
+        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
+        <v/>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C55" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H8,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D55" s="13" t="n"/>
+      <c r="E55" s="13" t="n"/>
+      <c r="F55" s="13">
+        <f>F54</f>
+        <v/>
+      </c>
+      <c r="H55" s="14">
+        <f>IF(ABS(F55-'Plan mensual'!K8)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7">
-        <f>'Plan mensual'!$A$9+21</f>
-        <v/>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="n"/>
-      <c r="E57" s="10">
-        <f>'Plan mensual'!J9</f>
-        <v/>
-      </c>
-      <c r="F57" s="9">
-        <f>F56+D57-E57</f>
-        <v/>
-      </c>
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Febrero 2027</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="6" t="n"/>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="6" t="n"/>
+      <c r="F57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <f>'Plan mensual'!$A$9-1</f>
         <v/>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D58" s="9" t="n"/>
-      <c r="E58" s="9">
-        <f>Supuestos!$B$29</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D58" s="10">
+        <f>'Plan mensual'!C9</f>
+        <v/>
+      </c>
+      <c r="E58" s="9" t="n"/>
       <c r="F58" s="9">
-        <f>F57+D58-E58</f>
+        <f>F55+D58-E58</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <f>'Plan mensual'!$A$9+14</f>
         <v/>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D59" s="9" t="n"/>
-      <c r="E59" s="9">
-        <f>Supuestos!$B$30</f>
+      <c r="E59" s="10">
+        <f>'Plan mensual'!F9</f>
         <v/>
       </c>
       <c r="F59" s="9">
@@ -1784,22 +1784,22 @@
     </row>
     <row r="60">
       <c r="A60" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <f>'Plan mensual'!$A$9+14</f>
         <v/>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D60" s="9" t="n"/>
-      <c r="E60" s="9">
-        <f>Supuestos!$B$31</f>
+      <c r="E60" s="10">
+        <f>'Plan mensual'!G9</f>
         <v/>
       </c>
       <c r="F60" s="9">
@@ -1809,22 +1809,22 @@
     </row>
     <row r="61">
       <c r="A61" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <f>'Plan mensual'!$A$9+21</f>
         <v/>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D61" s="9" t="n"/>
-      <c r="E61" s="9">
-        <f>Supuestos!$B$32</f>
+      <c r="E61" s="10">
+        <f>'Plan mensual'!J9</f>
         <v/>
       </c>
       <c r="F61" s="9">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="D62" s="9" t="n"/>
       <c r="E62" s="9">
-        <f>Supuestos!$B$33</f>
+        <f>Supuestos!$B$31</f>
         <v/>
       </c>
       <c r="F62" s="9">
@@ -1858,85 +1858,123 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="11">
+      <c r="A63" s="7">
         <f>EOMONTH('Plan mensual'!$A$9,0)</f>
         <v/>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C63" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H9,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D63" s="13" t="n"/>
-      <c r="E63" s="13" t="n"/>
-      <c r="F63" s="13">
-        <f>F62</f>
-        <v/>
-      </c>
-      <c r="H63" s="14">
-        <f>IF(ABS(F63-'Plan mensual'!K9)&lt;0.01,"OK","Revisar")</f>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Delivery (total del mes)</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="n"/>
+      <c r="E63" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
+      <c r="F63" s="9">
+        <f>F62+D63-E63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7">
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <v/>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>Taxis (total del mes)</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="n"/>
+      <c r="E64" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
+      <c r="F64" s="9">
+        <f>F63+D64-E64</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>Marzo 2027</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="6" t="n"/>
-      <c r="D65" s="6" t="n"/>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="6" t="n"/>
+      <c r="A65" s="7">
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <v/>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Otros (total del mes)</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="n"/>
+      <c r="E65" s="9">
+        <f>Supuestos!$B$34</f>
+        <v/>
+      </c>
+      <c r="F65" s="9">
+        <f>F64+D65-E65</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="7">
-        <f>'Plan mensual'!$A$10-1</f>
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
         <v/>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D66" s="10">
-        <f>'Plan mensual'!C10</f>
-        <v/>
-      </c>
-      <c r="E66" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="n"/>
+      <c r="E66" s="9">
+        <f>Supuestos!$B$35</f>
+        <v/>
+      </c>
       <c r="F66" s="9">
-        <f>F63+D66-E66</f>
+        <f>F65+D66-E66</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7">
-        <f>'Plan mensual'!$A$10+14</f>
+        <f>'Plan mensual'!$A$9+9</f>
         <v/>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D67" s="9" t="n"/>
-      <c r="E67" s="10">
-        <f>'Plan mensual'!F10</f>
+      <c r="E67" s="9">
+        <f>IF('Plan mensual'!$A$9&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F67" s="9">
@@ -1945,123 +1983,85 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7">
-        <f>'Plan mensual'!$A$10+14</f>
-        <v/>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>Cuota ExtraCash</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D68" s="9" t="n"/>
-      <c r="E68" s="10">
-        <f>'Plan mensual'!G10</f>
-        <v/>
-      </c>
-      <c r="F68" s="9">
-        <f>F67+D68-E68</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="7">
-        <f>'Plan mensual'!$A$10+21</f>
-        <v/>
-      </c>
-      <c r="B69" s="8" t="inlineStr">
-        <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D69" s="9" t="n"/>
-      <c r="E69" s="10">
-        <f>'Plan mensual'!J10</f>
-        <v/>
-      </c>
-      <c r="F69" s="9">
-        <f>F68+D69-E69</f>
+      <c r="A68" s="11">
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <v/>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C68" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H9,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D68" s="13" t="n"/>
+      <c r="E68" s="13" t="n"/>
+      <c r="F68" s="13">
+        <f>F67</f>
+        <v/>
+      </c>
+      <c r="H68" s="14">
+        <f>IF(ABS(F68-'Plan mensual'!K9)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
-        <v/>
-      </c>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>Supermercado (total del mes)</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D70" s="9" t="n"/>
-      <c r="E70" s="9">
-        <f>Supuestos!$B$29</f>
-        <v/>
-      </c>
-      <c r="F70" s="9">
-        <f>F69+D70-E70</f>
-        <v/>
-      </c>
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Marzo 2027</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="6" t="n"/>
+      <c r="D70" s="6" t="n"/>
+      <c r="E70" s="6" t="n"/>
+      <c r="F70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <f>'Plan mensual'!$A$10-1</f>
         <v/>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D71" s="9" t="n"/>
-      <c r="E71" s="9">
-        <f>Supuestos!$B$30</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D71" s="10">
+        <f>'Plan mensual'!C10</f>
+        <v/>
+      </c>
+      <c r="E71" s="9" t="n"/>
       <c r="F71" s="9">
-        <f>F70+D71-E71</f>
+        <f>F68+D71-E71</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <f>'Plan mensual'!$A$10+14</f>
         <v/>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D72" s="9" t="n"/>
-      <c r="E72" s="9">
-        <f>Supuestos!$B$31</f>
+      <c r="E72" s="10">
+        <f>'Plan mensual'!F10</f>
         <v/>
       </c>
       <c r="F72" s="9">
@@ -2071,22 +2071,22 @@
     </row>
     <row r="73">
       <c r="A73" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <f>'Plan mensual'!$A$10+14</f>
         <v/>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D73" s="9" t="n"/>
-      <c r="E73" s="9">
-        <f>Supuestos!$B$32</f>
+      <c r="E73" s="10">
+        <f>'Plan mensual'!G10</f>
         <v/>
       </c>
       <c r="F73" s="9">
@@ -2096,22 +2096,22 @@
     </row>
     <row r="74">
       <c r="A74" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <f>'Plan mensual'!$A$10+21</f>
         <v/>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D74" s="9" t="n"/>
-      <c r="E74" s="9">
-        <f>Supuestos!$B$33</f>
+      <c r="E74" s="10">
+        <f>'Plan mensual'!J10</f>
         <v/>
       </c>
       <c r="F74" s="9">
@@ -2120,85 +2120,123 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="11">
+      <c r="A75" s="7">
         <f>EOMONTH('Plan mensual'!$A$10,0)</f>
         <v/>
       </c>
-      <c r="B75" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C75" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H10,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D75" s="13" t="n"/>
-      <c r="E75" s="13" t="n"/>
-      <c r="F75" s="13">
-        <f>F74</f>
-        <v/>
-      </c>
-      <c r="H75" s="14">
-        <f>IF(ABS(F75-'Plan mensual'!K10)&lt;0.01,"OK","Revisar")</f>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado (total del mes)</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="n"/>
+      <c r="E75" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
+      <c r="F75" s="9">
+        <f>F74+D75-E75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7">
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <v/>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>Delivery (total del mes)</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="n"/>
+      <c r="E76" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
+      <c r="F76" s="9">
+        <f>F75+D76-E76</f>
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="inlineStr">
-        <is>
-          <t>Abril 2027</t>
-        </is>
-      </c>
-      <c r="B77" s="6" t="n"/>
-      <c r="C77" s="6" t="n"/>
-      <c r="D77" s="6" t="n"/>
-      <c r="E77" s="6" t="n"/>
-      <c r="F77" s="6" t="n"/>
+      <c r="A77" s="7">
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <v/>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>Taxis (total del mes)</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="n"/>
+      <c r="E77" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
+      <c r="F77" s="9">
+        <f>F76+D77-E77</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="7">
-        <f>'Plan mensual'!$A$11-1</f>
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
         <v/>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D78" s="10">
-        <f>'Plan mensual'!C11</f>
-        <v/>
-      </c>
-      <c r="E78" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="n"/>
+      <c r="E78" s="9">
+        <f>Supuestos!$B$34</f>
+        <v/>
+      </c>
       <c r="F78" s="9">
-        <f>F75+D78-E78</f>
+        <f>F77+D78-E78</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="7">
-        <f>'Plan mensual'!$A$11+14</f>
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
         <v/>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D79" s="9" t="n"/>
-      <c r="E79" s="10">
-        <f>'Plan mensual'!F11</f>
+      <c r="E79" s="9">
+        <f>Supuestos!$B$35</f>
         <v/>
       </c>
       <c r="F79" s="9">
@@ -2208,22 +2246,22 @@
     </row>
     <row r="80">
       <c r="A80" s="7">
-        <f>'Plan mensual'!$A$11+14</f>
+        <f>'Plan mensual'!$A$10+9</f>
         <v/>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D80" s="9" t="n"/>
-      <c r="E80" s="10">
-        <f>'Plan mensual'!G11</f>
+      <c r="E80" s="9">
+        <f>IF('Plan mensual'!$A$10&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F80" s="9">
@@ -2232,123 +2270,85 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="7">
-        <f>'Plan mensual'!$A$11+21</f>
-        <v/>
-      </c>
-      <c r="B81" s="8" t="inlineStr">
-        <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D81" s="9" t="n"/>
-      <c r="E81" s="10">
-        <f>'Plan mensual'!J11</f>
-        <v/>
-      </c>
-      <c r="F81" s="9">
-        <f>F80+D81-E81</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
-        <v/>
-      </c>
-      <c r="B82" s="8" t="inlineStr">
-        <is>
-          <t>Supermercado (total del mes)</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D82" s="9" t="n"/>
-      <c r="E82" s="9">
-        <f>Supuestos!$B$29</f>
-        <v/>
-      </c>
-      <c r="F82" s="9">
-        <f>F81+D82-E82</f>
+      <c r="A81" s="11">
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <v/>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C81" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H10,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D81" s="13" t="n"/>
+      <c r="E81" s="13" t="n"/>
+      <c r="F81" s="13">
+        <f>F80</f>
+        <v/>
+      </c>
+      <c r="H81" s="14">
+        <f>IF(ABS(F81-'Plan mensual'!K10)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
-        <v/>
-      </c>
-      <c r="B83" s="8" t="inlineStr">
-        <is>
-          <t>Delivery (total del mes)</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D83" s="9" t="n"/>
-      <c r="E83" s="9">
-        <f>Supuestos!$B$30</f>
-        <v/>
-      </c>
-      <c r="F83" s="9">
-        <f>F82+D83-E83</f>
-        <v/>
-      </c>
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Abril 2027</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
+      <c r="E83" s="6" t="n"/>
+      <c r="F83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <f>'Plan mensual'!$A$11-1</f>
         <v/>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D84" s="9" t="n"/>
-      <c r="E84" s="9">
-        <f>Supuestos!$B$31</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D84" s="10">
+        <f>'Plan mensual'!C11</f>
+        <v/>
+      </c>
+      <c r="E84" s="9" t="n"/>
       <c r="F84" s="9">
-        <f>F83+D84-E84</f>
+        <f>F81+D84-E84</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <f>'Plan mensual'!$A$11+14</f>
         <v/>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D85" s="9" t="n"/>
-      <c r="E85" s="9">
-        <f>Supuestos!$B$32</f>
+      <c r="E85" s="10">
+        <f>'Plan mensual'!F11</f>
         <v/>
       </c>
       <c r="F85" s="9">
@@ -2358,22 +2358,22 @@
     </row>
     <row r="86">
       <c r="A86" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <f>'Plan mensual'!$A$11+14</f>
         <v/>
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D86" s="9" t="n"/>
-      <c r="E86" s="9">
-        <f>Supuestos!$B$33</f>
+      <c r="E86" s="10">
+        <f>'Plan mensual'!G11</f>
         <v/>
       </c>
       <c r="F86" s="9">
@@ -2382,85 +2382,123 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="11">
+      <c r="A87" s="7">
+        <f>'Plan mensual'!$A$11+21</f>
+        <v/>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Prepago ExtraCash (reducir plazo)</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="n"/>
+      <c r="E87" s="10">
+        <f>'Plan mensual'!J11</f>
+        <v/>
+      </c>
+      <c r="F87" s="9">
+        <f>F86+D87-E87</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7">
         <f>EOMONTH('Plan mensual'!$A$11,0)</f>
         <v/>
       </c>
-      <c r="B87" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C87" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H11,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D87" s="13" t="n"/>
-      <c r="E87" s="13" t="n"/>
-      <c r="F87" s="13">
-        <f>F86</f>
-        <v/>
-      </c>
-      <c r="H87" s="14">
-        <f>IF(ABS(F87-'Plan mensual'!K11)&lt;0.01,"OK","Revisar")</f>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado (total del mes)</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="n"/>
+      <c r="E88" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
+      <c r="F88" s="9">
+        <f>F87+D88-E88</f>
         <v/>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="inlineStr">
-        <is>
-          <t>Mayo 2027</t>
-        </is>
-      </c>
-      <c r="B89" s="6" t="n"/>
-      <c r="C89" s="6" t="n"/>
-      <c r="D89" s="6" t="n"/>
-      <c r="E89" s="6" t="n"/>
-      <c r="F89" s="6" t="n"/>
+      <c r="A89" s="7">
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <v/>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Delivery (total del mes)</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="n"/>
+      <c r="E89" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
+      <c r="F89" s="9">
+        <f>F88+D89-E89</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="7">
-        <f>'Plan mensual'!$A$12-1</f>
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
         <v/>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D90" s="10">
-        <f>'Plan mensual'!C12</f>
-        <v/>
-      </c>
-      <c r="E90" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="n"/>
+      <c r="E90" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
       <c r="F90" s="9">
-        <f>F87+D90-E90</f>
+        <f>F89+D90-E90</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="7">
-        <f>'Plan mensual'!$A$12+14</f>
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
         <v/>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D91" s="9" t="n"/>
-      <c r="E91" s="10">
-        <f>'Plan mensual'!F12</f>
+      <c r="E91" s="9">
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F91" s="9">
@@ -2470,22 +2508,22 @@
     </row>
     <row r="92">
       <c r="A92" s="7">
-        <f>'Plan mensual'!$A$12+14</f>
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
         <v/>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D92" s="9" t="n"/>
-      <c r="E92" s="10">
-        <f>'Plan mensual'!G12</f>
+      <c r="E92" s="9">
+        <f>Supuestos!$B$35</f>
         <v/>
       </c>
       <c r="F92" s="9">
@@ -2495,22 +2533,22 @@
     </row>
     <row r="93">
       <c r="A93" s="7">
-        <f>'Plan mensual'!$A$12+21</f>
+        <f>'Plan mensual'!$A$11+9</f>
         <v/>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D93" s="9" t="n"/>
-      <c r="E93" s="10">
-        <f>'Plan mensual'!J12</f>
+      <c r="E93" s="9">
+        <f>IF('Plan mensual'!$A$11&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F93" s="9">
@@ -2519,123 +2557,85 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
-        <v/>
-      </c>
-      <c r="B94" s="8" t="inlineStr">
-        <is>
-          <t>Supermercado (total del mes)</t>
-        </is>
-      </c>
-      <c r="C94" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D94" s="9" t="n"/>
-      <c r="E94" s="9">
-        <f>Supuestos!$B$29</f>
-        <v/>
-      </c>
-      <c r="F94" s="9">
-        <f>F93+D94-E94</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
-        <v/>
-      </c>
-      <c r="B95" s="8" t="inlineStr">
-        <is>
-          <t>Delivery (total del mes)</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D95" s="9" t="n"/>
-      <c r="E95" s="9">
-        <f>Supuestos!$B$30</f>
-        <v/>
-      </c>
-      <c r="F95" s="9">
-        <f>F94+D95-E95</f>
+      <c r="A94" s="11">
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <v/>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C94" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H11,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D94" s="13" t="n"/>
+      <c r="E94" s="13" t="n"/>
+      <c r="F94" s="13">
+        <f>F93</f>
+        <v/>
+      </c>
+      <c r="H94" s="14">
+        <f>IF(ABS(F94-'Plan mensual'!K11)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
-        <v/>
-      </c>
-      <c r="B96" s="8" t="inlineStr">
-        <is>
-          <t>Taxis (total del mes)</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D96" s="9" t="n"/>
-      <c r="E96" s="9">
-        <f>Supuestos!$B$31</f>
-        <v/>
-      </c>
-      <c r="F96" s="9">
-        <f>F95+D96-E96</f>
-        <v/>
-      </c>
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>Mayo 2027</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="n"/>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="6" t="n"/>
+      <c r="F96" s="6" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <f>'Plan mensual'!$A$12-1</f>
         <v/>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D97" s="9" t="n"/>
-      <c r="E97" s="9">
-        <f>Supuestos!$B$32</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D97" s="10">
+        <f>'Plan mensual'!C12</f>
+        <v/>
+      </c>
+      <c r="E97" s="9" t="n"/>
       <c r="F97" s="9">
-        <f>F96+D97-E97</f>
+        <f>F94+D97-E97</f>
         <v/>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <f>'Plan mensual'!$A$12+14</f>
         <v/>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D98" s="9" t="n"/>
-      <c r="E98" s="9">
-        <f>Supuestos!$B$33</f>
+      <c r="E98" s="10">
+        <f>'Plan mensual'!F12</f>
         <v/>
       </c>
       <c r="F98" s="9">
@@ -2644,85 +2644,123 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="11">
+      <c r="A99" s="7">
+        <f>'Plan mensual'!$A$12+14</f>
+        <v/>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Cuota ExtraCash</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="n"/>
+      <c r="E99" s="10">
+        <f>'Plan mensual'!G12</f>
+        <v/>
+      </c>
+      <c r="F99" s="9">
+        <f>F98+D99-E99</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7">
+        <f>'Plan mensual'!$A$12+21</f>
+        <v/>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>Prepago ExtraCash (reducir plazo)</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="n"/>
+      <c r="E100" s="10">
+        <f>'Plan mensual'!J12</f>
+        <v/>
+      </c>
+      <c r="F100" s="9">
+        <f>F99+D100-E100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="7">
         <f>EOMONTH('Plan mensual'!$A$12,0)</f>
         <v/>
       </c>
-      <c r="B99" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C99" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H12,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D99" s="13" t="n"/>
-      <c r="E99" s="13" t="n"/>
-      <c r="F99" s="13">
-        <f>F98</f>
-        <v/>
-      </c>
-      <c r="H99" s="14">
-        <f>IF(ABS(F99-'Plan mensual'!K12)&lt;0.01,"OK","Revisar")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>Junio 2027</t>
-        </is>
-      </c>
-      <c r="B101" s="6" t="n"/>
-      <c r="C101" s="6" t="n"/>
-      <c r="D101" s="6" t="n"/>
-      <c r="E101" s="6" t="n"/>
-      <c r="F101" s="6" t="n"/>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado (total del mes)</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="n"/>
+      <c r="E101" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
+      <c r="F101" s="9">
+        <f>F100+D101-E101</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="7">
-        <f>'Plan mensual'!$A$13-1</f>
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
         <v/>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Delivery (total del mes)</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D102" s="10">
-        <f>'Plan mensual'!C13</f>
-        <v/>
-      </c>
-      <c r="E102" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="n"/>
+      <c r="E102" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
       <c r="F102" s="9">
-        <f>F99+D102-E102</f>
+        <f>F101+D102-E102</f>
         <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="7">
-        <f>'Plan mensual'!$A$13+14</f>
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
         <v/>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D103" s="9" t="n"/>
-      <c r="E103" s="10">
-        <f>'Plan mensual'!F13</f>
+      <c r="E103" s="9">
+        <f>Supuestos!$B$33</f>
         <v/>
       </c>
       <c r="F103" s="9">
@@ -2732,22 +2770,22 @@
     </row>
     <row r="104">
       <c r="A104" s="7">
-        <f>'Plan mensual'!$A$13+14</f>
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
         <v/>
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D104" s="9" t="n"/>
-      <c r="E104" s="10">
-        <f>'Plan mensual'!G13</f>
+      <c r="E104" s="9">
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F104" s="9">
@@ -2757,22 +2795,22 @@
     </row>
     <row r="105">
       <c r="A105" s="7">
-        <f>'Plan mensual'!$A$13+21</f>
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
         <v/>
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D105" s="9" t="n"/>
-      <c r="E105" s="10">
-        <f>'Plan mensual'!J13</f>
+      <c r="E105" s="9">
+        <f>Supuestos!$B$35</f>
         <v/>
       </c>
       <c r="F105" s="9">
@@ -2782,22 +2820,22 @@
     </row>
     <row r="106">
       <c r="A106" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <f>'Plan mensual'!$A$12+9</f>
         <v/>
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D106" s="9" t="n"/>
       <c r="E106" s="9">
-        <f>Supuestos!$B$29</f>
+        <f>IF('Plan mensual'!$A$12&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F106" s="9">
@@ -2806,127 +2844,314 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B107" s="8" t="inlineStr">
-        <is>
-          <t>Delivery (total del mes)</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D107" s="9" t="n"/>
-      <c r="E107" s="9">
-        <f>Supuestos!$B$30</f>
-        <v/>
-      </c>
-      <c r="F107" s="9">
-        <f>F106+D107-E107</f>
-        <v/>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B108" s="8" t="inlineStr">
-        <is>
-          <t>Taxis (total del mes)</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D108" s="9" t="n"/>
-      <c r="E108" s="9">
-        <f>Supuestos!$B$31</f>
-        <v/>
-      </c>
-      <c r="F108" s="9">
-        <f>F107+D108-E108</f>
+      <c r="A107" s="11">
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <v/>
+      </c>
+      <c r="B107" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C107" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H12,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D107" s="13" t="n"/>
+      <c r="E107" s="13" t="n"/>
+      <c r="F107" s="13">
+        <f>F106</f>
+        <v/>
+      </c>
+      <c r="H107" s="14">
+        <f>IF(ABS(F107-'Plan mensual'!K12)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B109" s="8" t="inlineStr">
-        <is>
-          <t>Otros (total del mes)</t>
-        </is>
-      </c>
-      <c r="C109" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D109" s="9" t="n"/>
-      <c r="E109" s="9">
-        <f>Supuestos!$B$32</f>
-        <v/>
-      </c>
-      <c r="F109" s="9">
-        <f>F108+D109-E109</f>
-        <v/>
-      </c>
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>Junio 2027</t>
+        </is>
+      </c>
+      <c r="B109" s="6" t="n"/>
+      <c r="C109" s="6" t="n"/>
+      <c r="D109" s="6" t="n"/>
+      <c r="E109" s="6" t="n"/>
+      <c r="F109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="7">
+        <f>'Plan mensual'!$A$13-1</f>
+        <v/>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>Sueldo Simtryx</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D110" s="10">
+        <f>'Plan mensual'!C13</f>
+        <v/>
+      </c>
+      <c r="E110" s="9" t="n"/>
+      <c r="F110" s="9">
+        <f>F107+D110-E110</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="7">
+        <f>'Plan mensual'!$A$13+14</f>
+        <v/>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="n"/>
+      <c r="E111" s="10">
+        <f>'Plan mensual'!F13</f>
+        <v/>
+      </c>
+      <c r="F111" s="9">
+        <f>F110+D111-E111</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="7">
+        <f>'Plan mensual'!$A$13+14</f>
+        <v/>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>Cuota ExtraCash</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="n"/>
+      <c r="E112" s="10">
+        <f>'Plan mensual'!G13</f>
+        <v/>
+      </c>
+      <c r="F112" s="9">
+        <f>F111+D112-E112</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="7">
+        <f>'Plan mensual'!$A$13+21</f>
+        <v/>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>Prepago ExtraCash (reducir plazo)</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="n"/>
+      <c r="E113" s="10">
+        <f>'Plan mensual'!J13</f>
+        <v/>
+      </c>
+      <c r="F113" s="9">
+        <f>F112+D113-E113</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7">
         <f>EOMONTH('Plan mensual'!$A$13,0)</f>
         <v/>
       </c>
-      <c r="B110" s="8" t="inlineStr">
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado (total del mes)</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="n"/>
+      <c r="E114" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
+      <c r="F114" s="9">
+        <f>F113+D114-E114</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7">
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <v/>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>Delivery (total del mes)</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="n"/>
+      <c r="E115" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
+      <c r="F115" s="9">
+        <f>F114+D115-E115</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7">
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <v/>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>Taxis (total del mes)</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="n"/>
+      <c r="E116" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
+      <c r="F116" s="9">
+        <f>F115+D116-E116</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="7">
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <v/>
+      </c>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t>Otros (total del mes)</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="n"/>
+      <c r="E117" s="9">
+        <f>Supuestos!$B$34</f>
+        <v/>
+      </c>
+      <c r="F117" s="9">
+        <f>F116+D117-E117</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7">
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <v/>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
         <is>
           <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
-      <c r="C110" s="8" t="inlineStr">
+      <c r="C118" s="8" t="inlineStr">
         <is>
           <t>Gasto de vida</t>
         </is>
       </c>
-      <c r="D110" s="9" t="n"/>
-      <c r="E110" s="9">
-        <f>Supuestos!$B$33</f>
-        <v/>
-      </c>
-      <c r="F110" s="9">
-        <f>F109+D110-E110</f>
-        <v/>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="11">
+      <c r="D118" s="9" t="n"/>
+      <c r="E118" s="9">
+        <f>Supuestos!$B$35</f>
+        <v/>
+      </c>
+      <c r="F118" s="9">
+        <f>F117+D118-E118</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7">
+        <f>'Plan mensual'!$A$13+9</f>
+        <v/>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>Mantenimiento + agua (Yape)</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>Gasto fijo</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="n"/>
+      <c r="E119" s="9">
+        <f>IF('Plan mensual'!$A$13&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <v/>
+      </c>
+      <c r="F119" s="9">
+        <f>F118+D119-E119</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="11">
         <f>EOMONTH('Plan mensual'!$A$13,0)</f>
         <v/>
       </c>
-      <c r="B111" s="12" t="inlineStr">
+      <c r="B120" s="12" t="inlineStr">
         <is>
           <t>SALDO FINAL DEL MES</t>
         </is>
       </c>
-      <c r="C111" s="12">
+      <c r="C120" s="12">
         <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H13,"#,##0.00")</f>
         <v/>
       </c>
-      <c r="D111" s="13" t="n"/>
-      <c r="E111" s="13" t="n"/>
-      <c r="F111" s="13">
-        <f>F110</f>
-        <v/>
-      </c>
-      <c r="H111" s="14">
-        <f>IF(ABS(F111-'Plan mensual'!K13)&lt;0.01,"OK","Revisar")</f>
+      <c r="D120" s="13" t="n"/>
+      <c r="E120" s="13" t="n"/>
+      <c r="F120" s="13">
+        <f>F119</f>
+        <v/>
+      </c>
+      <c r="H120" s="14">
+        <f>IF(ABS(F120-'Plan mensual'!K13)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
@@ -2941,7 +3166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -3279,119 +3504,149 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Mantenimiento + agua del edificio (débito)</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n">
+        <v>197</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Usuario 11/10/2026: se paga cada mes hasta diciembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Último mes de mantenimiento</t>
+        </is>
+      </c>
+      <c r="B28" s="24" t="n">
+        <v>46357</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Usuario: hasta diciembre (mudanza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Gastos de vida con débito (mes completo)</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n"/>
-      <c r="C27" s="16" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="25" t="inlineStr">
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
         <is>
           <t>Rubro</t>
         </is>
       </c>
-      <c r="B28" s="25" t="inlineStr">
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>Mes completo</t>
         </is>
       </c>
-      <c r="C28" s="25" t="inlineStr">
+      <c r="C30" s="25" t="inlineStr">
         <is>
           <t>Octubre (desde el 05/10)</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>Supermercado</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="C29" s="18" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
-        <is>
-          <t>Delivery</t>
-        </is>
-      </c>
-      <c r="B30" s="18" t="n">
-        <v>300</v>
-      </c>
-      <c r="C30" s="18" t="n">
-        <v>225</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>Taxis</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="B31" s="18" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="C31" s="18" t="n">
-        <v>225</v>
+        <v>400</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="B32" s="18" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C32" s="18" t="n">
-        <v>120</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
+          <t>Taxis</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="C34" s="18" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
           <t>Contador Luxr</t>
         </is>
       </c>
-      <c r="B33" s="18" t="n">
+      <c r="B35" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="C33" s="18" t="n">
+      <c r="C35" s="18" t="n">
         <v>150</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Notas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>- Regla: la tarjeta solo carga servicios fijos y se paga completa el 15 del mes siguiente.</t>
-        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>- Cada mes se aparta en caja lo cargado a la tarjeta ese mes. El resto va a prepago (reducir plazo).</t>
+          <t>Notas:</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>- Regla: la tarjeta solo carga servicios fijos y se paga completa el 15 del mes siguiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>- Cada mes se aparta en caja lo cargado a la tarjeta ese mes. El resto va a prepago (reducir plazo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>- El interés del ExtraCash se aproxima con TEM sobre el saldo de inicio de mes.</t>
         </is>
@@ -3543,7 +3798,7 @@
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>Supuestos!$C$29+Supuestos!$C$30+Supuestos!$C$31+Supuestos!$C$32+Supuestos!$C$33</f>
+        <f>Supuestos!$C$31+Supuestos!$C$32+Supuestos!$C$33+Supuestos!$C$34+Supuestos!$C$35+IF(A5&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F5" s="10">
@@ -3609,7 +3864,7 @@
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A6&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F6" s="9">
@@ -3675,7 +3930,7 @@
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A7&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F7" s="9">
@@ -3741,7 +3996,7 @@
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A8&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F8" s="9">
@@ -3807,7 +4062,7 @@
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A9&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F9" s="9">
@@ -3873,7 +4128,7 @@
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A10&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F10" s="9">
@@ -3939,7 +4194,7 @@
         <v/>
       </c>
       <c r="E11" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A11&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F11" s="9">
@@ -4005,7 +4260,7 @@
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A12&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F12" s="9">
@@ -4071,7 +4326,7 @@
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A13&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F13" s="9">

</xml_diff>

<commit_message>
Remove delivery from debt ledger budget
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EPNKNk7kASs5DQVTsUv5rh
</commit_message>
<xml_diff>
--- a/finanzas/libro-caja-deuda.xlsx
+++ b/finanzas/libro-caja-deuda.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -786,22 +786,22 @@
     </row>
     <row r="14">
       <c r="A14" s="7">
-        <f>EOMONTH('Plan mensual'!$A$5,0)</f>
+        <f>'Plan mensual'!$A$5+9</f>
         <v/>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9">
-        <f>Supuestos!$C$35</f>
+        <f>IF('Plan mensual'!$A$5&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F14" s="9">
@@ -810,89 +810,89 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7">
-        <f>'Plan mensual'!$A$5+9</f>
-        <v/>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Mantenimiento + agua (Yape)</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9">
-        <f>IF('Plan mensual'!$A$5&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="9">
-        <f>F14+D15-E15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11">
+      <c r="A15" s="11">
         <f>EOMONTH('Plan mensual'!$A$5,0)</f>
         <v/>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>SALDO FINAL DEL MES</t>
         </is>
       </c>
-      <c r="C16" s="12">
+      <c r="C15" s="12">
         <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H5,"#,##0.00")</f>
         <v/>
       </c>
-      <c r="D16" s="13" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13">
-        <f>F15</f>
-        <v/>
-      </c>
-      <c r="H16" s="14">
-        <f>IF(ABS(F16-'Plan mensual'!K5)&lt;0.01,"OK","Revisar")</f>
-        <v/>
-      </c>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13">
+        <f>F14</f>
+        <v/>
+      </c>
+      <c r="H15" s="14">
+        <f>IF(ABS(F15-'Plan mensual'!K5)&lt;0.01,"OK","Revisar")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Noviembre 2026</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Noviembre 2026</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
+      <c r="A18" s="7">
+        <f>'Plan mensual'!$A$6-1</f>
+        <v/>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Sueldo Simtryx</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D18" s="10">
+        <f>'Plan mensual'!C6</f>
+        <v/>
+      </c>
+      <c r="E18" s="9" t="n"/>
+      <c r="F18" s="9">
+        <f>F15+D18-E18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7">
-        <f>'Plan mensual'!$A$6-1</f>
+        <f>'Plan mensual'!$A$6+14</f>
         <v/>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior) + pendientes + interés residual</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D19" s="10">
-        <f>'Plan mensual'!C6</f>
-        <v/>
-      </c>
-      <c r="E19" s="9" t="n"/>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="10">
+        <f>'Plan mensual'!F6</f>
+        <v/>
+      </c>
       <c r="F19" s="9">
-        <f>F16+D19-E19</f>
+        <f>F18+D19-E19</f>
         <v/>
       </c>
     </row>
@@ -903,17 +903,17 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior) + pendientes + interés residual</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="10">
-        <f>'Plan mensual'!F6</f>
+        <f>'Plan mensual'!G6</f>
         <v/>
       </c>
       <c r="F20" s="9">
@@ -923,12 +923,12 @@
     </row>
     <row r="21">
       <c r="A21" s="7">
-        <f>'Plan mensual'!$A$6+14</f>
+        <f>'Plan mensual'!$A$6+21</f>
         <v/>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="10">
-        <f>'Plan mensual'!G6</f>
+        <f>'Plan mensual'!J6</f>
         <v/>
       </c>
       <c r="F21" s="9">
@@ -948,22 +948,22 @@
     </row>
     <row r="22">
       <c r="A22" s="7">
-        <f>'Plan mensual'!$A$6+21</f>
+        <f>EOMONTH('Plan mensual'!$A$6,0)</f>
         <v/>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D22" s="9" t="n"/>
-      <c r="E22" s="10">
-        <f>'Plan mensual'!J6</f>
+      <c r="E22" s="9">
+        <f>Supuestos!$B$31</f>
         <v/>
       </c>
       <c r="F22" s="9">
@@ -978,7 +978,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9">
-        <f>Supuestos!$B$31</f>
+        <f>Supuestos!$B$32</f>
         <v/>
       </c>
       <c r="F23" s="9">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9">
-        <f>Supuestos!$B$32</f>
+        <f>Supuestos!$B$33</f>
         <v/>
       </c>
       <c r="F24" s="9">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9">
-        <f>Supuestos!$B$33</f>
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F25" s="9">
@@ -1048,22 +1048,22 @@
     </row>
     <row r="26">
       <c r="A26" s="7">
-        <f>EOMONTH('Plan mensual'!$A$6,0)</f>
+        <f>'Plan mensual'!$A$6+9</f>
         <v/>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9">
-        <f>Supuestos!$B$34</f>
+        <f>IF('Plan mensual'!$A$6&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F26" s="9">
@@ -1072,135 +1072,135 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7">
+      <c r="A27" s="11">
         <f>EOMONTH('Plan mensual'!$A$6,0)</f>
         <v/>
       </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Contador Luxr (total del mes)</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="9">
-        <f>Supuestos!$B$35</f>
-        <v/>
-      </c>
-      <c r="F27" s="9">
-        <f>F26+D27-E27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7">
-        <f>'Plan mensual'!$A$6+9</f>
-        <v/>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>Mantenimiento + agua (Yape)</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9">
-        <f>IF('Plan mensual'!$A$6&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
-        <v/>
-      </c>
-      <c r="F28" s="9">
-        <f>F27+D28-E28</f>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C27" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H6,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13">
+        <f>F26</f>
+        <v/>
+      </c>
+      <c r="H27" s="14">
+        <f>IF(ABS(F27-'Plan mensual'!K6)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11">
-        <f>EOMONTH('Plan mensual'!$A$6,0)</f>
-        <v/>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C29" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H6,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13">
-        <f>F28</f>
-        <v/>
-      </c>
-      <c r="H29" s="14">
-        <f>IF(ABS(F29-'Plan mensual'!K6)&lt;0.01,"OK","Revisar")</f>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Diciembre 2026</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7">
+        <f>'Plan mensual'!$A$7-1</f>
+        <v/>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Sueldo Simtryx</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D30" s="10">
+        <f>'Plan mensual'!C7</f>
+        <v/>
+      </c>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="9">
+        <f>F27+D30-E30</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Diciembre 2026</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
+      <c r="A31" s="7">
+        <f>'Plan mensual'!$A$7+14</f>
+        <v/>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="10">
+        <f>'Plan mensual'!F7</f>
+        <v/>
+      </c>
+      <c r="F31" s="9">
+        <f>F30+D31-E31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7">
-        <f>'Plan mensual'!$A$7-1</f>
+        <f>'Plan mensual'!$A$7+14</f>
         <v/>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D32" s="10">
-        <f>'Plan mensual'!C7</f>
-        <v/>
-      </c>
-      <c r="E32" s="9" t="n"/>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="10">
+        <f>'Plan mensual'!G7</f>
+        <v/>
+      </c>
       <c r="F32" s="9">
-        <f>F29+D32-E32</f>
+        <f>F31+D32-E32</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7">
-        <f>'Plan mensual'!$A$7+14</f>
+        <f>'Plan mensual'!$A$7+21</f>
         <v/>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="10">
-        <f>'Plan mensual'!F7</f>
+        <f>'Plan mensual'!J7</f>
         <v/>
       </c>
       <c r="F33" s="9">
@@ -1210,22 +1210,22 @@
     </row>
     <row r="34">
       <c r="A34" s="7">
-        <f>'Plan mensual'!$A$7+14</f>
+        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
         <v/>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D34" s="9" t="n"/>
-      <c r="E34" s="10">
-        <f>'Plan mensual'!G7</f>
+      <c r="E34" s="9">
+        <f>Supuestos!$B$31</f>
         <v/>
       </c>
       <c r="F34" s="9">
@@ -1235,22 +1235,22 @@
     </row>
     <row r="35">
       <c r="A35" s="7">
-        <f>'Plan mensual'!$A$7+21</f>
+        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
         <v/>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D35" s="9" t="n"/>
-      <c r="E35" s="10">
-        <f>'Plan mensual'!J7</f>
+      <c r="E35" s="9">
+        <f>Supuestos!$B$32</f>
         <v/>
       </c>
       <c r="F35" s="9">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="9">
-        <f>Supuestos!$B$31</f>
+        <f>Supuestos!$B$33</f>
         <v/>
       </c>
       <c r="F36" s="9">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="9">
-        <f>Supuestos!$B$32</f>
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F37" s="9">
@@ -1310,22 +1310,22 @@
     </row>
     <row r="38">
       <c r="A38" s="7">
-        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
+        <f>'Plan mensual'!$A$7+9</f>
         <v/>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D38" s="9" t="n"/>
       <c r="E38" s="9">
-        <f>Supuestos!$B$33</f>
+        <f>IF('Plan mensual'!$A$7&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F38" s="9">
@@ -1334,160 +1334,160 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7">
+      <c r="A39" s="11">
         <f>EOMONTH('Plan mensual'!$A$7,0)</f>
         <v/>
       </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>Otros (total del mes)</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="n"/>
-      <c r="E39" s="9">
-        <f>Supuestos!$B$34</f>
-        <v/>
-      </c>
-      <c r="F39" s="9">
-        <f>F38+D39-E39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7">
-        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
-        <v/>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>Contador Luxr (total del mes)</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="n"/>
-      <c r="E40" s="9">
-        <f>Supuestos!$B$35</f>
-        <v/>
-      </c>
-      <c r="F40" s="9">
-        <f>F39+D40-E40</f>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C39" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H7,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D39" s="13" t="n"/>
+      <c r="E39" s="13" t="n"/>
+      <c r="F39" s="13">
+        <f>F38</f>
+        <v/>
+      </c>
+      <c r="H39" s="14">
+        <f>IF(ABS(F39-'Plan mensual'!K7)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7">
-        <f>'Plan mensual'!$A$7+9</f>
-        <v/>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>Mantenimiento + agua (Yape)</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="n"/>
-      <c r="E41" s="9">
-        <f>IF('Plan mensual'!$A$7&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
-        <v/>
-      </c>
-      <c r="F41" s="9">
-        <f>F40+D41-E41</f>
-        <v/>
-      </c>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Enero 2027</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="11">
-        <f>EOMONTH('Plan mensual'!$A$7,0)</f>
-        <v/>
-      </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C42" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H7,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D42" s="13" t="n"/>
-      <c r="E42" s="13" t="n"/>
-      <c r="F42" s="13">
-        <f>F41</f>
-        <v/>
-      </c>
-      <c r="H42" s="14">
-        <f>IF(ABS(F42-'Plan mensual'!K7)&lt;0.01,"OK","Revisar")</f>
+      <c r="A42" s="7">
+        <f>'Plan mensual'!$A$8-1</f>
+        <v/>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Sueldo Simtryx</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D42" s="10">
+        <f>'Plan mensual'!C8</f>
+        <v/>
+      </c>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="9">
+        <f>F39+D42-E42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7">
+        <f>'Plan mensual'!$A$8+14</f>
+        <v/>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="10">
+        <f>'Plan mensual'!F8</f>
+        <v/>
+      </c>
+      <c r="F43" s="9">
+        <f>F42+D43-E43</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Enero 2027</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="6" t="n"/>
-      <c r="D44" s="6" t="n"/>
-      <c r="E44" s="6" t="n"/>
-      <c r="F44" s="6" t="n"/>
+      <c r="A44" s="7">
+        <f>'Plan mensual'!$A$8+14</f>
+        <v/>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Cuota ExtraCash</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="10">
+        <f>'Plan mensual'!G8</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>F43+D44-E44</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7">
-        <f>'Plan mensual'!$A$8-1</f>
+        <f>'Plan mensual'!$A$8+21</f>
         <v/>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D45" s="10">
-        <f>'Plan mensual'!C8</f>
-        <v/>
-      </c>
-      <c r="E45" s="9" t="n"/>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="10">
+        <f>'Plan mensual'!J8</f>
+        <v/>
+      </c>
       <c r="F45" s="9">
-        <f>F42+D45-E45</f>
+        <f>F44+D45-E45</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7">
-        <f>'Plan mensual'!$A$8+14</f>
+        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
         <v/>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D46" s="9" t="n"/>
-      <c r="E46" s="10">
-        <f>'Plan mensual'!F8</f>
+      <c r="E46" s="9">
+        <f>Supuestos!$B$31</f>
         <v/>
       </c>
       <c r="F46" s="9">
@@ -1497,22 +1497,22 @@
     </row>
     <row r="47">
       <c r="A47" s="7">
-        <f>'Plan mensual'!$A$8+14</f>
+        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
         <v/>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D47" s="9" t="n"/>
-      <c r="E47" s="10">
-        <f>'Plan mensual'!G8</f>
+      <c r="E47" s="9">
+        <f>Supuestos!$B$32</f>
         <v/>
       </c>
       <c r="F47" s="9">
@@ -1522,22 +1522,22 @@
     </row>
     <row r="48">
       <c r="A48" s="7">
-        <f>'Plan mensual'!$A$8+21</f>
+        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
         <v/>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D48" s="9" t="n"/>
-      <c r="E48" s="10">
-        <f>'Plan mensual'!J8</f>
+      <c r="E48" s="9">
+        <f>Supuestos!$B$33</f>
         <v/>
       </c>
       <c r="F48" s="9">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="9">
-        <f>Supuestos!$B$31</f>
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F49" s="9">
@@ -1572,22 +1572,22 @@
     </row>
     <row r="50">
       <c r="A50" s="7">
-        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
+        <f>'Plan mensual'!$A$8+9</f>
         <v/>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D50" s="9" t="n"/>
       <c r="E50" s="9">
-        <f>Supuestos!$B$32</f>
+        <f>IF('Plan mensual'!$A$8&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F50" s="9">
@@ -1596,185 +1596,185 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7">
+      <c r="A51" s="11">
         <f>EOMONTH('Plan mensual'!$A$8,0)</f>
         <v/>
       </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>Taxis (total del mes)</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9">
-        <f>Supuestos!$B$33</f>
-        <v/>
-      </c>
-      <c r="F51" s="9">
-        <f>F50+D51-E51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7">
-        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
-        <v/>
-      </c>
-      <c r="B52" s="8" t="inlineStr">
-        <is>
-          <t>Otros (total del mes)</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="n"/>
-      <c r="E52" s="9">
-        <f>Supuestos!$B$34</f>
-        <v/>
-      </c>
-      <c r="F52" s="9">
-        <f>F51+D52-E52</f>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C51" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H8,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D51" s="13" t="n"/>
+      <c r="E51" s="13" t="n"/>
+      <c r="F51" s="13">
+        <f>F50</f>
+        <v/>
+      </c>
+      <c r="H51" s="14">
+        <f>IF(ABS(F51-'Plan mensual'!K8)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7">
-        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
-        <v/>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>Contador Luxr (total del mes)</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="n"/>
-      <c r="E53" s="9">
-        <f>Supuestos!$B$35</f>
-        <v/>
-      </c>
-      <c r="F53" s="9">
-        <f>F52+D53-E53</f>
-        <v/>
-      </c>
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Febrero 2027</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7">
-        <f>'Plan mensual'!$A$8+9</f>
+        <f>'Plan mensual'!$A$9-1</f>
         <v/>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Mantenimiento + agua (Yape)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="n"/>
-      <c r="E54" s="9">
-        <f>IF('Plan mensual'!$A$8&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D54" s="10">
+        <f>'Plan mensual'!C9</f>
+        <v/>
+      </c>
+      <c r="E54" s="9" t="n"/>
       <c r="F54" s="9">
-        <f>F53+D54-E54</f>
+        <f>F51+D54-E54</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="11">
-        <f>EOMONTH('Plan mensual'!$A$8,0)</f>
-        <v/>
-      </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C55" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H8,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D55" s="13" t="n"/>
-      <c r="E55" s="13" t="n"/>
-      <c r="F55" s="13">
-        <f>F54</f>
-        <v/>
-      </c>
-      <c r="H55" s="14">
-        <f>IF(ABS(F55-'Plan mensual'!K8)&lt;0.01,"OK","Revisar")</f>
+      <c r="A55" s="7">
+        <f>'Plan mensual'!$A$9+14</f>
+        <v/>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="n"/>
+      <c r="E55" s="10">
+        <f>'Plan mensual'!F9</f>
+        <v/>
+      </c>
+      <c r="F55" s="9">
+        <f>F54+D55-E55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7">
+        <f>'Plan mensual'!$A$9+14</f>
+        <v/>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>Cuota ExtraCash</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="n"/>
+      <c r="E56" s="10">
+        <f>'Plan mensual'!G9</f>
+        <v/>
+      </c>
+      <c r="F56" s="9">
+        <f>F55+D56-E56</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>Febrero 2027</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="6" t="n"/>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="6" t="n"/>
+      <c r="A57" s="7">
+        <f>'Plan mensual'!$A$9+21</f>
+        <v/>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Prepago ExtraCash (reducir plazo)</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="n"/>
+      <c r="E57" s="10">
+        <f>'Plan mensual'!J9</f>
+        <v/>
+      </c>
+      <c r="F57" s="9">
+        <f>F56+D57-E57</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7">
-        <f>'Plan mensual'!$A$9-1</f>
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
         <v/>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D58" s="10">
-        <f>'Plan mensual'!C9</f>
-        <v/>
-      </c>
-      <c r="E58" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="n"/>
+      <c r="E58" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
       <c r="F58" s="9">
-        <f>F55+D58-E58</f>
+        <f>F57+D58-E58</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7">
-        <f>'Plan mensual'!$A$9+14</f>
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
         <v/>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D59" s="9" t="n"/>
-      <c r="E59" s="10">
-        <f>'Plan mensual'!F9</f>
+      <c r="E59" s="9">
+        <f>Supuestos!$B$32</f>
         <v/>
       </c>
       <c r="F59" s="9">
@@ -1784,22 +1784,22 @@
     </row>
     <row r="60">
       <c r="A60" s="7">
-        <f>'Plan mensual'!$A$9+14</f>
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
         <v/>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D60" s="9" t="n"/>
-      <c r="E60" s="10">
-        <f>'Plan mensual'!G9</f>
+      <c r="E60" s="9">
+        <f>Supuestos!$B$33</f>
         <v/>
       </c>
       <c r="F60" s="9">
@@ -1809,22 +1809,22 @@
     </row>
     <row r="61">
       <c r="A61" s="7">
-        <f>'Plan mensual'!$A$9+21</f>
+        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
         <v/>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D61" s="9" t="n"/>
-      <c r="E61" s="10">
-        <f>'Plan mensual'!J9</f>
+      <c r="E61" s="9">
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F61" s="9">
@@ -1834,22 +1834,22 @@
     </row>
     <row r="62">
       <c r="A62" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <f>'Plan mensual'!$A$9+9</f>
         <v/>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Supermercado (total del mes)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D62" s="9" t="n"/>
       <c r="E62" s="9">
-        <f>Supuestos!$B$31</f>
+        <f>IF('Plan mensual'!$A$9&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F62" s="9">
@@ -1858,123 +1858,85 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7">
+      <c r="A63" s="11">
         <f>EOMONTH('Plan mensual'!$A$9,0)</f>
         <v/>
       </c>
-      <c r="B63" s="8" t="inlineStr">
-        <is>
-          <t>Delivery (total del mes)</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D63" s="9" t="n"/>
-      <c r="E63" s="9">
-        <f>Supuestos!$B$32</f>
-        <v/>
-      </c>
-      <c r="F63" s="9">
-        <f>F62+D63-E63</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
-        <v/>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>Taxis (total del mes)</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D64" s="9" t="n"/>
-      <c r="E64" s="9">
-        <f>Supuestos!$B$33</f>
-        <v/>
-      </c>
-      <c r="F64" s="9">
-        <f>F63+D64-E64</f>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C63" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H9,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D63" s="13" t="n"/>
+      <c r="E63" s="13" t="n"/>
+      <c r="F63" s="13">
+        <f>F62</f>
+        <v/>
+      </c>
+      <c r="H63" s="14">
+        <f>IF(ABS(F63-'Plan mensual'!K9)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
-        <v/>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>Otros (total del mes)</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="n"/>
-      <c r="E65" s="9">
-        <f>Supuestos!$B$34</f>
-        <v/>
-      </c>
-      <c r="F65" s="9">
-        <f>F64+D65-E65</f>
-        <v/>
-      </c>
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Marzo 2027</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
+        <f>'Plan mensual'!$A$10-1</f>
         <v/>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D66" s="9" t="n"/>
-      <c r="E66" s="9">
-        <f>Supuestos!$B$35</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D66" s="10">
+        <f>'Plan mensual'!C10</f>
+        <v/>
+      </c>
+      <c r="E66" s="9" t="n"/>
       <c r="F66" s="9">
-        <f>F65+D66-E66</f>
+        <f>F63+D66-E66</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7">
-        <f>'Plan mensual'!$A$9+9</f>
+        <f>'Plan mensual'!$A$10+14</f>
         <v/>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Mantenimiento + agua (Yape)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Gasto fijo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D67" s="9" t="n"/>
-      <c r="E67" s="9">
-        <f>IF('Plan mensual'!$A$9&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+      <c r="E67" s="10">
+        <f>'Plan mensual'!F10</f>
         <v/>
       </c>
       <c r="F67" s="9">
@@ -1983,85 +1945,123 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="11">
-        <f>EOMONTH('Plan mensual'!$A$9,0)</f>
-        <v/>
-      </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C68" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H9,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D68" s="13" t="n"/>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="13">
-        <f>F67</f>
-        <v/>
-      </c>
-      <c r="H68" s="14">
-        <f>IF(ABS(F68-'Plan mensual'!K9)&lt;0.01,"OK","Revisar")</f>
+      <c r="A68" s="7">
+        <f>'Plan mensual'!$A$10+14</f>
+        <v/>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>Cuota ExtraCash</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="n"/>
+      <c r="E68" s="10">
+        <f>'Plan mensual'!G10</f>
+        <v/>
+      </c>
+      <c r="F68" s="9">
+        <f>F67+D68-E68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7">
+        <f>'Plan mensual'!$A$10+21</f>
+        <v/>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>Prepago ExtraCash (reducir plazo)</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="n"/>
+      <c r="E69" s="10">
+        <f>'Plan mensual'!J10</f>
+        <v/>
+      </c>
+      <c r="F69" s="9">
+        <f>F68+D69-E69</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>Marzo 2027</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="n"/>
-      <c r="C70" s="6" t="n"/>
-      <c r="D70" s="6" t="n"/>
-      <c r="E70" s="6" t="n"/>
-      <c r="F70" s="6" t="n"/>
+      <c r="A70" s="7">
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <v/>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado (total del mes)</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="n"/>
+      <c r="E70" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
+      <c r="F70" s="9">
+        <f>F69+D70-E70</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="7">
-        <f>'Plan mensual'!$A$10-1</f>
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
         <v/>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Taxis (total del mes)</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D71" s="10">
-        <f>'Plan mensual'!C10</f>
-        <v/>
-      </c>
-      <c r="E71" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="n"/>
+      <c r="E71" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
       <c r="F71" s="9">
-        <f>F68+D71-E71</f>
+        <f>F70+D71-E71</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7">
-        <f>'Plan mensual'!$A$10+14</f>
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
         <v/>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D72" s="9" t="n"/>
-      <c r="E72" s="10">
-        <f>'Plan mensual'!F10</f>
+      <c r="E72" s="9">
+        <f>Supuestos!$B$33</f>
         <v/>
       </c>
       <c r="F72" s="9">
@@ -2071,22 +2071,22 @@
     </row>
     <row r="73">
       <c r="A73" s="7">
-        <f>'Plan mensual'!$A$10+14</f>
+        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
         <v/>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D73" s="9" t="n"/>
-      <c r="E73" s="10">
-        <f>'Plan mensual'!G10</f>
+      <c r="E73" s="9">
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F73" s="9">
@@ -2096,22 +2096,22 @@
     </row>
     <row r="74">
       <c r="A74" s="7">
-        <f>'Plan mensual'!$A$10+21</f>
+        <f>'Plan mensual'!$A$10+9</f>
         <v/>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D74" s="9" t="n"/>
-      <c r="E74" s="10">
-        <f>'Plan mensual'!J10</f>
+      <c r="E74" s="9">
+        <f>IF('Plan mensual'!$A$10&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F74" s="9">
@@ -2120,123 +2120,85 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="7">
+      <c r="A75" s="11">
         <f>EOMONTH('Plan mensual'!$A$10,0)</f>
         <v/>
       </c>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>Supermercado (total del mes)</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D75" s="9" t="n"/>
-      <c r="E75" s="9">
-        <f>Supuestos!$B$31</f>
-        <v/>
-      </c>
-      <c r="F75" s="9">
-        <f>F74+D75-E75</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
-        <v/>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>Delivery (total del mes)</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D76" s="9" t="n"/>
-      <c r="E76" s="9">
-        <f>Supuestos!$B$32</f>
-        <v/>
-      </c>
-      <c r="F76" s="9">
-        <f>F75+D76-E76</f>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C75" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H10,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D75" s="13" t="n"/>
+      <c r="E75" s="13" t="n"/>
+      <c r="F75" s="13">
+        <f>F74</f>
+        <v/>
+      </c>
+      <c r="H75" s="14">
+        <f>IF(ABS(F75-'Plan mensual'!K10)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
-        <v/>
-      </c>
-      <c r="B77" s="8" t="inlineStr">
-        <is>
-          <t>Taxis (total del mes)</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D77" s="9" t="n"/>
-      <c r="E77" s="9">
-        <f>Supuestos!$B$33</f>
-        <v/>
-      </c>
-      <c r="F77" s="9">
-        <f>F76+D77-E77</f>
-        <v/>
-      </c>
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Abril 2027</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
+      <c r="F77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <f>'Plan mensual'!$A$11-1</f>
         <v/>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D78" s="9" t="n"/>
-      <c r="E78" s="9">
-        <f>Supuestos!$B$34</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D78" s="10">
+        <f>'Plan mensual'!C11</f>
+        <v/>
+      </c>
+      <c r="E78" s="9" t="n"/>
       <c r="F78" s="9">
-        <f>F77+D78-E78</f>
+        <f>F75+D78-E78</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="7">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
+        <f>'Plan mensual'!$A$11+14</f>
         <v/>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D79" s="9" t="n"/>
-      <c r="E79" s="9">
-        <f>Supuestos!$B$35</f>
+      <c r="E79" s="10">
+        <f>'Plan mensual'!F11</f>
         <v/>
       </c>
       <c r="F79" s="9">
@@ -2246,22 +2208,22 @@
     </row>
     <row r="80">
       <c r="A80" s="7">
-        <f>'Plan mensual'!$A$10+9</f>
+        <f>'Plan mensual'!$A$11+14</f>
         <v/>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Mantenimiento + agua (Yape)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Gasto fijo</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D80" s="9" t="n"/>
-      <c r="E80" s="9">
-        <f>IF('Plan mensual'!$A$10&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+      <c r="E80" s="10">
+        <f>'Plan mensual'!G11</f>
         <v/>
       </c>
       <c r="F80" s="9">
@@ -2270,85 +2232,123 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="11">
-        <f>EOMONTH('Plan mensual'!$A$10,0)</f>
-        <v/>
-      </c>
-      <c r="B81" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C81" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H10,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D81" s="13" t="n"/>
-      <c r="E81" s="13" t="n"/>
-      <c r="F81" s="13">
-        <f>F80</f>
-        <v/>
-      </c>
-      <c r="H81" s="14">
-        <f>IF(ABS(F81-'Plan mensual'!K10)&lt;0.01,"OK","Revisar")</f>
+      <c r="A81" s="7">
+        <f>'Plan mensual'!$A$11+21</f>
+        <v/>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Prepago ExtraCash (reducir plazo)</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Deuda</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="n"/>
+      <c r="E81" s="10">
+        <f>'Plan mensual'!J11</f>
+        <v/>
+      </c>
+      <c r="F81" s="9">
+        <f>F80+D81-E81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7">
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <v/>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado (total del mes)</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="n"/>
+      <c r="E82" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
+      <c r="F82" s="9">
+        <f>F81+D82-E82</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="inlineStr">
-        <is>
-          <t>Abril 2027</t>
-        </is>
-      </c>
-      <c r="B83" s="6" t="n"/>
-      <c r="C83" s="6" t="n"/>
-      <c r="D83" s="6" t="n"/>
-      <c r="E83" s="6" t="n"/>
-      <c r="F83" s="6" t="n"/>
+      <c r="A83" s="7">
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <v/>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>Taxis (total del mes)</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="n"/>
+      <c r="E83" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
+      <c r="F83" s="9">
+        <f>F82+D83-E83</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="7">
-        <f>'Plan mensual'!$A$11-1</f>
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
         <v/>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Otros (total del mes)</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D84" s="10">
-        <f>'Plan mensual'!C11</f>
-        <v/>
-      </c>
-      <c r="E84" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="n"/>
+      <c r="E84" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
       <c r="F84" s="9">
-        <f>F81+D84-E84</f>
+        <f>F83+D84-E84</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="7">
-        <f>'Plan mensual'!$A$11+14</f>
+        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
         <v/>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D85" s="9" t="n"/>
-      <c r="E85" s="10">
-        <f>'Plan mensual'!F11</f>
+      <c r="E85" s="9">
+        <f>Supuestos!$B$34</f>
         <v/>
       </c>
       <c r="F85" s="9">
@@ -2358,22 +2358,22 @@
     </row>
     <row r="86">
       <c r="A86" s="7">
-        <f>'Plan mensual'!$A$11+14</f>
+        <f>'Plan mensual'!$A$11+9</f>
         <v/>
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>Cuota ExtraCash</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D86" s="9" t="n"/>
-      <c r="E86" s="10">
-        <f>'Plan mensual'!G11</f>
+      <c r="E86" s="9">
+        <f>IF('Plan mensual'!$A$11&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F86" s="9">
@@ -2382,123 +2382,85 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="7">
-        <f>'Plan mensual'!$A$11+21</f>
-        <v/>
-      </c>
-      <c r="B87" s="8" t="inlineStr">
-        <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D87" s="9" t="n"/>
-      <c r="E87" s="10">
-        <f>'Plan mensual'!J11</f>
-        <v/>
-      </c>
-      <c r="F87" s="9">
-        <f>F86+D87-E87</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="7">
+      <c r="A87" s="11">
         <f>EOMONTH('Plan mensual'!$A$11,0)</f>
         <v/>
       </c>
-      <c r="B88" s="8" t="inlineStr">
-        <is>
-          <t>Supermercado (total del mes)</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D88" s="9" t="n"/>
-      <c r="E88" s="9">
-        <f>Supuestos!$B$31</f>
-        <v/>
-      </c>
-      <c r="F88" s="9">
-        <f>F87+D88-E88</f>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C87" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H11,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D87" s="13" t="n"/>
+      <c r="E87" s="13" t="n"/>
+      <c r="F87" s="13">
+        <f>F86</f>
+        <v/>
+      </c>
+      <c r="H87" s="14">
+        <f>IF(ABS(F87-'Plan mensual'!K11)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
-        <v/>
-      </c>
-      <c r="B89" s="8" t="inlineStr">
-        <is>
-          <t>Delivery (total del mes)</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D89" s="9" t="n"/>
-      <c r="E89" s="9">
-        <f>Supuestos!$B$32</f>
-        <v/>
-      </c>
-      <c r="F89" s="9">
-        <f>F88+D89-E89</f>
-        <v/>
-      </c>
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>Mayo 2027</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="6" t="n"/>
+      <c r="F89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <f>'Plan mensual'!$A$12-1</f>
         <v/>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D90" s="9" t="n"/>
-      <c r="E90" s="9">
-        <f>Supuestos!$B$33</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D90" s="10">
+        <f>'Plan mensual'!C12</f>
+        <v/>
+      </c>
+      <c r="E90" s="9" t="n"/>
       <c r="F90" s="9">
-        <f>F89+D90-E90</f>
+        <f>F87+D90-E90</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <f>'Plan mensual'!$A$12+14</f>
         <v/>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D91" s="9" t="n"/>
-      <c r="E91" s="9">
-        <f>Supuestos!$B$34</f>
+      <c r="E91" s="10">
+        <f>'Plan mensual'!F12</f>
         <v/>
       </c>
       <c r="F91" s="9">
@@ -2508,22 +2470,22 @@
     </row>
     <row r="92">
       <c r="A92" s="7">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
+        <f>'Plan mensual'!$A$12+14</f>
         <v/>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D92" s="9" t="n"/>
-      <c r="E92" s="9">
-        <f>Supuestos!$B$35</f>
+      <c r="E92" s="10">
+        <f>'Plan mensual'!G12</f>
         <v/>
       </c>
       <c r="F92" s="9">
@@ -2533,22 +2495,22 @@
     </row>
     <row r="93">
       <c r="A93" s="7">
-        <f>'Plan mensual'!$A$11+9</f>
+        <f>'Plan mensual'!$A$12+21</f>
         <v/>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Mantenimiento + agua (Yape)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Gasto fijo</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D93" s="9" t="n"/>
-      <c r="E93" s="9">
-        <f>IF('Plan mensual'!$A$11&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+      <c r="E93" s="10">
+        <f>'Plan mensual'!J12</f>
         <v/>
       </c>
       <c r="F93" s="9">
@@ -2557,85 +2519,123 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="11">
-        <f>EOMONTH('Plan mensual'!$A$11,0)</f>
-        <v/>
-      </c>
-      <c r="B94" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C94" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H11,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D94" s="13" t="n"/>
-      <c r="E94" s="13" t="n"/>
-      <c r="F94" s="13">
-        <f>F93</f>
-        <v/>
-      </c>
-      <c r="H94" s="14">
-        <f>IF(ABS(F94-'Plan mensual'!K11)&lt;0.01,"OK","Revisar")</f>
+      <c r="A94" s="7">
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <v/>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>Supermercado (total del mes)</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D94" s="9" t="n"/>
+      <c r="E94" s="9">
+        <f>Supuestos!$B$31</f>
+        <v/>
+      </c>
+      <c r="F94" s="9">
+        <f>F93+D94-E94</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7">
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <v/>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>Taxis (total del mes)</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="n"/>
+      <c r="E95" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
+      <c r="F95" s="9">
+        <f>F94+D95-E95</f>
         <v/>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Mayo 2027</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="n"/>
-      <c r="C96" s="6" t="n"/>
-      <c r="D96" s="6" t="n"/>
-      <c r="E96" s="6" t="n"/>
-      <c r="F96" s="6" t="n"/>
+      <c r="A96" s="7">
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <v/>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>Otros (total del mes)</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="n"/>
+      <c r="E96" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
+      <c r="F96" s="9">
+        <f>F95+D96-E96</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="7">
-        <f>'Plan mensual'!$A$12-1</f>
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
         <v/>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Contador Luxr (total del mes)</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D97" s="10">
-        <f>'Plan mensual'!C12</f>
-        <v/>
-      </c>
-      <c r="E97" s="9" t="n"/>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="n"/>
+      <c r="E97" s="9">
+        <f>Supuestos!$B$34</f>
+        <v/>
+      </c>
       <c r="F97" s="9">
-        <f>F94+D97-E97</f>
+        <f>F96+D97-E97</f>
         <v/>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="7">
-        <f>'Plan mensual'!$A$12+14</f>
+        <f>'Plan mensual'!$A$12+9</f>
         <v/>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Gasto fijo</t>
         </is>
       </c>
       <c r="D98" s="9" t="n"/>
-      <c r="E98" s="10">
-        <f>'Plan mensual'!F12</f>
+      <c r="E98" s="9">
+        <f>IF('Plan mensual'!$A$12&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F98" s="9">
@@ -2644,123 +2644,85 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="7">
-        <f>'Plan mensual'!$A$12+14</f>
-        <v/>
-      </c>
-      <c r="B99" s="8" t="inlineStr">
-        <is>
-          <t>Cuota ExtraCash</t>
-        </is>
-      </c>
-      <c r="C99" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D99" s="9" t="n"/>
-      <c r="E99" s="10">
-        <f>'Plan mensual'!G12</f>
-        <v/>
-      </c>
-      <c r="F99" s="9">
-        <f>F98+D99-E99</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="7">
-        <f>'Plan mensual'!$A$12+21</f>
-        <v/>
-      </c>
-      <c r="B100" s="8" t="inlineStr">
-        <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
-        </is>
-      </c>
-      <c r="C100" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D100" s="9" t="n"/>
-      <c r="E100" s="10">
-        <f>'Plan mensual'!J12</f>
-        <v/>
-      </c>
-      <c r="F100" s="9">
-        <f>F99+D100-E100</f>
+      <c r="A99" s="11">
+        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <v/>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>SALDO FINAL DEL MES</t>
+        </is>
+      </c>
+      <c r="C99" s="12">
+        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H12,"#,##0.00")</f>
+        <v/>
+      </c>
+      <c r="D99" s="13" t="n"/>
+      <c r="E99" s="13" t="n"/>
+      <c r="F99" s="13">
+        <f>F98</f>
+        <v/>
+      </c>
+      <c r="H99" s="14">
+        <f>IF(ABS(F99-'Plan mensual'!K12)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
-        <v/>
-      </c>
-      <c r="B101" s="8" t="inlineStr">
-        <is>
-          <t>Supermercado (total del mes)</t>
-        </is>
-      </c>
-      <c r="C101" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D101" s="9" t="n"/>
-      <c r="E101" s="9">
-        <f>Supuestos!$B$31</f>
-        <v/>
-      </c>
-      <c r="F101" s="9">
-        <f>F100+D101-E101</f>
-        <v/>
-      </c>
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Junio 2027</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="n"/>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="6" t="n"/>
+      <c r="F101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <f>'Plan mensual'!$A$13-1</f>
         <v/>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>Delivery (total del mes)</t>
+          <t>Sueldo Simtryx</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D102" s="9" t="n"/>
-      <c r="E102" s="9">
-        <f>Supuestos!$B$32</f>
-        <v/>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="D102" s="10">
+        <f>'Plan mensual'!C13</f>
+        <v/>
+      </c>
+      <c r="E102" s="9" t="n"/>
       <c r="F102" s="9">
-        <f>F101+D102-E102</f>
+        <f>F99+D102-E102</f>
         <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <f>'Plan mensual'!$A$13+14</f>
         <v/>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Taxis (total del mes)</t>
+          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Tarjeta</t>
         </is>
       </c>
       <c r="D103" s="9" t="n"/>
-      <c r="E103" s="9">
-        <f>Supuestos!$B$33</f>
+      <c r="E103" s="10">
+        <f>'Plan mensual'!F13</f>
         <v/>
       </c>
       <c r="F103" s="9">
@@ -2770,22 +2732,22 @@
     </row>
     <row r="104">
       <c r="A104" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <f>'Plan mensual'!$A$13+14</f>
         <v/>
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>Otros (total del mes)</t>
+          <t>Cuota ExtraCash</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D104" s="9" t="n"/>
-      <c r="E104" s="9">
-        <f>Supuestos!$B$34</f>
+      <c r="E104" s="10">
+        <f>'Plan mensual'!G13</f>
         <v/>
       </c>
       <c r="F104" s="9">
@@ -2795,22 +2757,22 @@
     </row>
     <row r="105">
       <c r="A105" s="7">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
+        <f>'Plan mensual'!$A$13+21</f>
         <v/>
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>Contador Luxr (total del mes)</t>
+          <t>Prepago ExtraCash (reducir plazo)</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Gasto de vida</t>
+          <t>Deuda</t>
         </is>
       </c>
       <c r="D105" s="9" t="n"/>
-      <c r="E105" s="9">
-        <f>Supuestos!$B$35</f>
+      <c r="E105" s="10">
+        <f>'Plan mensual'!J13</f>
         <v/>
       </c>
       <c r="F105" s="9">
@@ -2820,22 +2782,22 @@
     </row>
     <row r="106">
       <c r="A106" s="7">
-        <f>'Plan mensual'!$A$12+9</f>
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
         <v/>
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>Mantenimiento + agua (Yape)</t>
+          <t>Supermercado (total del mes)</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>Gasto fijo</t>
+          <t>Gasto de vida</t>
         </is>
       </c>
       <c r="D106" s="9" t="n"/>
       <c r="E106" s="9">
-        <f>IF('Plan mensual'!$A$12&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31</f>
         <v/>
       </c>
       <c r="F106" s="9">
@@ -2844,314 +2806,127 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="11">
-        <f>EOMONTH('Plan mensual'!$A$12,0)</f>
-        <v/>
-      </c>
-      <c r="B107" s="12" t="inlineStr">
-        <is>
-          <t>SALDO FINAL DEL MES</t>
-        </is>
-      </c>
-      <c r="C107" s="12">
-        <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H12,"#,##0.00")</f>
-        <v/>
-      </c>
-      <c r="D107" s="13" t="n"/>
-      <c r="E107" s="13" t="n"/>
-      <c r="F107" s="13">
-        <f>F106</f>
-        <v/>
-      </c>
-      <c r="H107" s="14">
-        <f>IF(ABS(F107-'Plan mensual'!K12)&lt;0.01,"OK","Revisar")</f>
+      <c r="A107" s="7">
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <v/>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>Taxis (total del mes)</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="n"/>
+      <c r="E107" s="9">
+        <f>Supuestos!$B$32</f>
+        <v/>
+      </c>
+      <c r="F107" s="9">
+        <f>F106+D107-E107</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="7">
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <v/>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>Otros (total del mes)</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="n"/>
+      <c r="E108" s="9">
+        <f>Supuestos!$B$33</f>
+        <v/>
+      </c>
+      <c r="F108" s="9">
+        <f>F107+D108-E108</f>
         <v/>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="inlineStr">
-        <is>
-          <t>Junio 2027</t>
-        </is>
-      </c>
-      <c r="B109" s="6" t="n"/>
-      <c r="C109" s="6" t="n"/>
-      <c r="D109" s="6" t="n"/>
-      <c r="E109" s="6" t="n"/>
-      <c r="F109" s="6" t="n"/>
+      <c r="A109" s="7">
+        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
+        <v/>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>Contador Luxr (total del mes)</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>Gasto de vida</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="n"/>
+      <c r="E109" s="9">
+        <f>Supuestos!$B$34</f>
+        <v/>
+      </c>
+      <c r="F109" s="9">
+        <f>F108+D109-E109</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="7">
-        <f>'Plan mensual'!$A$13-1</f>
+        <f>'Plan mensual'!$A$13+9</f>
         <v/>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>Sueldo Simtryx</t>
+          <t>Mantenimiento + agua (Yape)</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D110" s="10">
-        <f>'Plan mensual'!C13</f>
-        <v/>
-      </c>
-      <c r="E110" s="9" t="n"/>
+          <t>Gasto fijo</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="n"/>
+      <c r="E110" s="9">
+        <f>IF('Plan mensual'!$A$13&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <v/>
+      </c>
       <c r="F110" s="9">
-        <f>F107+D110-E110</f>
+        <f>F109+D110-E110</f>
         <v/>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="7">
-        <f>'Plan mensual'!$A$13+14</f>
-        <v/>
-      </c>
-      <c r="B111" s="8" t="inlineStr">
-        <is>
-          <t>Pago estado de cuenta tarjeta (cargos del mes anterior)</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="D111" s="9" t="n"/>
-      <c r="E111" s="10">
-        <f>'Plan mensual'!F13</f>
-        <v/>
-      </c>
-      <c r="F111" s="9">
-        <f>F110+D111-E111</f>
-        <v/>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="7">
-        <f>'Plan mensual'!$A$13+14</f>
-        <v/>
-      </c>
-      <c r="B112" s="8" t="inlineStr">
-        <is>
-          <t>Cuota ExtraCash</t>
-        </is>
-      </c>
-      <c r="C112" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D112" s="9" t="n"/>
-      <c r="E112" s="10">
-        <f>'Plan mensual'!G13</f>
-        <v/>
-      </c>
-      <c r="F112" s="9">
-        <f>F111+D112-E112</f>
-        <v/>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="7">
-        <f>'Plan mensual'!$A$13+21</f>
-        <v/>
-      </c>
-      <c r="B113" s="8" t="inlineStr">
-        <is>
-          <t>Prepago ExtraCash (reducir plazo)</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="inlineStr">
-        <is>
-          <t>Deuda</t>
-        </is>
-      </c>
-      <c r="D113" s="9" t="n"/>
-      <c r="E113" s="10">
-        <f>'Plan mensual'!J13</f>
-        <v/>
-      </c>
-      <c r="F113" s="9">
-        <f>F112+D113-E113</f>
-        <v/>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="7">
+      <c r="A111" s="11">
         <f>EOMONTH('Plan mensual'!$A$13,0)</f>
         <v/>
       </c>
-      <c r="B114" s="8" t="inlineStr">
-        <is>
-          <t>Supermercado (total del mes)</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D114" s="9" t="n"/>
-      <c r="E114" s="9">
-        <f>Supuestos!$B$31</f>
-        <v/>
-      </c>
-      <c r="F114" s="9">
-        <f>F113+D114-E114</f>
-        <v/>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B115" s="8" t="inlineStr">
-        <is>
-          <t>Delivery (total del mes)</t>
-        </is>
-      </c>
-      <c r="C115" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D115" s="9" t="n"/>
-      <c r="E115" s="9">
-        <f>Supuestos!$B$32</f>
-        <v/>
-      </c>
-      <c r="F115" s="9">
-        <f>F114+D115-E115</f>
-        <v/>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B116" s="8" t="inlineStr">
-        <is>
-          <t>Taxis (total del mes)</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D116" s="9" t="n"/>
-      <c r="E116" s="9">
-        <f>Supuestos!$B$33</f>
-        <v/>
-      </c>
-      <c r="F116" s="9">
-        <f>F115+D116-E116</f>
-        <v/>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B117" s="8" t="inlineStr">
-        <is>
-          <t>Otros (total del mes)</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D117" s="9" t="n"/>
-      <c r="E117" s="9">
-        <f>Supuestos!$B$34</f>
-        <v/>
-      </c>
-      <c r="F117" s="9">
-        <f>F116+D117-E117</f>
-        <v/>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="7">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B118" s="8" t="inlineStr">
-        <is>
-          <t>Contador Luxr (total del mes)</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t>Gasto de vida</t>
-        </is>
-      </c>
-      <c r="D118" s="9" t="n"/>
-      <c r="E118" s="9">
-        <f>Supuestos!$B$35</f>
-        <v/>
-      </c>
-      <c r="F118" s="9">
-        <f>F117+D118-E118</f>
-        <v/>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="7">
-        <f>'Plan mensual'!$A$13+9</f>
-        <v/>
-      </c>
-      <c r="B119" s="8" t="inlineStr">
-        <is>
-          <t>Mantenimiento + agua (Yape)</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>Gasto fijo</t>
-        </is>
-      </c>
-      <c r="D119" s="9" t="n"/>
-      <c r="E119" s="9">
-        <f>IF('Plan mensual'!$A$13&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
-        <v/>
-      </c>
-      <c r="F119" s="9">
-        <f>F118+D119-E119</f>
-        <v/>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="11">
-        <f>EOMONTH('Plan mensual'!$A$13,0)</f>
-        <v/>
-      </c>
-      <c r="B120" s="12" t="inlineStr">
+      <c r="B111" s="12" t="inlineStr">
         <is>
           <t>SALDO FINAL DEL MES</t>
         </is>
       </c>
-      <c r="C120" s="12">
+      <c r="C111" s="12">
         <f>"Apartado tarjeta: S/ "&amp;TEXT('Plan mensual'!H13,"#,##0.00")</f>
         <v/>
       </c>
-      <c r="D120" s="13" t="n"/>
-      <c r="E120" s="13" t="n"/>
-      <c r="F120" s="13">
-        <f>F119</f>
-        <v/>
-      </c>
-      <c r="H120" s="14">
-        <f>IF(ABS(F120-'Plan mensual'!K13)&lt;0.01,"OK","Revisar")</f>
+      <c r="D111" s="13" t="n"/>
+      <c r="E111" s="13" t="n"/>
+      <c r="F111" s="13">
+        <f>F110</f>
+        <v/>
+      </c>
+      <c r="H111" s="14">
+        <f>IF(ABS(F111-'Plan mensual'!K13)&lt;0.01,"OK","Revisar")</f>
         <v/>
       </c>
     </row>
@@ -3166,7 +2941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -3575,7 +3350,7 @@
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Taxis</t>
         </is>
       </c>
       <c r="B32" s="18" t="n">
@@ -3588,65 +3363,52 @@
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>Taxis</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B33" s="18" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C33" s="18" t="n">
-        <v>225</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Contador Luxr</t>
         </is>
       </c>
       <c r="B34" s="18" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C34" s="18" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>Contador Luxr</t>
-        </is>
-      </c>
-      <c r="B35" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="C35" s="18" t="n">
-        <v>150</v>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Notas:</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Notas:</t>
+          <t>- Regla: la tarjeta solo carga servicios fijos y se paga completa el 15 del mes siguiente.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>- Regla: la tarjeta solo carga servicios fijos y se paga completa el 15 del mes siguiente.</t>
+          <t>- Cada mes se aparta en caja lo cargado a la tarjeta ese mes. El resto va a prepago (reducir plazo).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>- Cada mes se aparta en caja lo cargado a la tarjeta ese mes. El resto va a prepago (reducir plazo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>- El interés del ExtraCash se aproxima con TEM sobre el saldo de inicio de mes.</t>
         </is>
@@ -3798,7 +3560,7 @@
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>Supuestos!$C$31+Supuestos!$C$32+Supuestos!$C$33+Supuestos!$C$34+Supuestos!$C$35+IF(A5&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$C$31+Supuestos!$C$32+Supuestos!$C$33+Supuestos!$C$34+IF(A5&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F5" s="10">
@@ -3864,7 +3626,7 @@
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A6&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A6&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F6" s="9">
@@ -3930,7 +3692,7 @@
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A7&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A7&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F7" s="9">
@@ -3996,7 +3758,7 @@
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A8&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A8&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F8" s="9">
@@ -4062,7 +3824,7 @@
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A9&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A9&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F9" s="9">
@@ -4128,7 +3890,7 @@
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A10&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A10&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F10" s="9">
@@ -4194,7 +3956,7 @@
         <v/>
       </c>
       <c r="E11" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A11&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A11&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F11" s="9">
@@ -4260,7 +4022,7 @@
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A12&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A12&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F12" s="9">
@@ -4326,7 +4088,7 @@
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+Supuestos!$B$35+IF(A13&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
+        <f>Supuestos!$B$31+Supuestos!$B$32+Supuestos!$B$33+Supuestos!$B$34+IF(A13&lt;=Supuestos!$B$28,Supuestos!$B$27,0)</f>
         <v/>
       </c>
       <c r="F13" s="9">

</xml_diff>